<commit_message>
sending message when the task pass correctly
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$I$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ABIIDI</t>
+          <t>ABIDI</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -719,8 +719,43 @@
         <v>4099.13</v>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>KADRI</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Nacer</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chef projet </t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>405.16</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1190.56</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>2817.78</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add the number of paiment file
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$J$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -553,36 +553,36 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ABIDI</t>
+          <t xml:space="preserve">BEN FARHAT </t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MED aziz</t>
+          <t>Ismail</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>developeur</t>
+          <t xml:space="preserve">responsable materielles </t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2900</v>
+        <v>2600</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>680</v>
+        <v>450</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>329.88</v>
+        <v>280.68</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>903.5599999999999</v>
+        <v>715.96</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2360.06</v>
+        <v>2060.86</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -633,36 +633,36 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BRAHMI</t>
+          <t>ABIDI</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Hamza</t>
+          <t>MED aziz</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">chef projet </t>
+          <t>developeur</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6000</v>
+        <v>2900</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1000</v>
+        <v>680</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>644.11</v>
+        <v>329.88</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2101.61</v>
+        <v>903.5599999999999</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4270.78</v>
+        <v>2360.06</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -673,36 +673,36 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEN FARHAT </t>
+          <t>BRAHMI</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Ismail</t>
+          <t>Hamza</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">responsable materielles </t>
+          <t xml:space="preserve">chef projet </t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2600</v>
+        <v>6000</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>450</v>
+        <v>1000</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>280.68</v>
+        <v>644.11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>715.96</v>
+        <v>2101.61</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>2060.86</v>
+        <v>4270.78</v>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
@@ -713,36 +713,36 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MASSMOUDI</t>
+          <t>KADRI</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Chaima</t>
+          <t>Nacer</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RH </t>
+          <t xml:space="preserve">chef projet </t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5400</v>
+        <v>6000</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>600</v>
+        <v>780</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>551.9</v>
+        <v>623.23</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1750.03</v>
+        <v>2021.98</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3710.07</v>
+        <v>4143.79</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -753,45 +753,245 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>KADRI</t>
+          <t>MASSMOUDI</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Nacer</t>
+          <t>Chaima</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">chef projet </t>
+          <t xml:space="preserve">RH </t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>6000</v>
+        <v>5400</v>
       </c>
       <c r="E7" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>551.9</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1750.03</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>3710.07</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>AL AZIZ</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>BILEL</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ingénieure de fonction</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>780</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>623.23</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>2021.98</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>4143.79</v>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="F8" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>301.93</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>796.98</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>2190.09</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>BEN ARFFA</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>BINEN</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>RH</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>5200</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>522.25</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>1636.98</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>3529.77</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>MOUSSA</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AHMED</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>developpeur</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>290</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>87.26000000000001</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>91.79000000000001</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>771.45</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>AJOULI</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ISSRA</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>ingénieure de production</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>312.81</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>838.46</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>2256.23</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HAWAWI</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>MOSTAFA</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">derecteur générale </t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>671.9299999999999</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>2207.66</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>4439.91</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Aout 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixing the number of file
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$J$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,19 +483,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -549,21 +550,26 @@
           <t>Periode</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Bulltein</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEN FARHAT </t>
+          <t>BEN FARHAT</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Ismail</t>
+          <t>ISMAIL</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">responsable materielles </t>
+          <t>responsable materielles</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -588,46 +594,52 @@
         <is>
           <t>Aout 2026</t>
         </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>BEN HASSEN</t>
+          <t>BEN HASEN</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Mariem</t>
+          <t>MARIEM</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">responsable logistique </t>
+          <t>responsable logistique</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>4000</v>
+        <v>2900</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>500</v>
+        <v>680</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>413.93</v>
+        <v>329.88</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>1223.98</v>
+        <v>903.5599999999999</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>2871.09</v>
+        <v>2360.06</v>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Aout 2026</t>
         </is>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -643,7 +655,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>developeur</t>
+          <t>developpeur</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -669,329 +681,12 @@
           <t>Aout 2026</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Hamza</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>644.11</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>2101.61</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>4270.78</v>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>KADRI</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Nacer</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>780</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>623.23</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>2021.98</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>4143.79</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>MASSMOUDI</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Chaima</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RH </t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>5400</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>600</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>551.9</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>1750.03</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>3710.07</v>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>AL AZIZ</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>BILEL</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>ingénieure de fonction</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>2900</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>301.93</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>796.98</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>2190.09</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>BEN ARFFA</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>BINEN</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>RH</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>5200</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>480</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>522.25</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>1636.98</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>3529.77</v>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>MOUSSA</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>AHMED</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>developpeur</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>290</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>650</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>87.26000000000001</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>91.79000000000001</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>771.45</v>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>AJOULI</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>ISSRA</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>ingénieure de production</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>400</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>312.81</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>838.46</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>2256.23</v>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>HAWAWI</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>MOSTAFA</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">derecteur générale </t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>6500</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>800</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>671.9299999999999</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>2207.66</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>4439.91</v>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
+      <c r="K4" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:K4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add a historie paiment file
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -110,6 +115,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -477,17 +494,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -595,8 +612,188 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>BRAHMI</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>HAMZA</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chef projet </t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>644.25</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>2102.13</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>4271.61</v>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>N°002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KADRI</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NACER</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cheft projet </t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>597.53</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1923.98</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>3987.49</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>N°003</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>BEN ISSA</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>MARIEM</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>RH</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>5800</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>670</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>594.91</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1914.01</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>3971.58</v>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>N°004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>AL AZIZ</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MOSTAFA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>RESPONSABLE LOGISTIQUE</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>465.75</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>1421.56</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>3186.19</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>N°005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
make a compare betwen two different paiment file for the same employee
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -792,8 +792,53 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>BRAHMI</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>HAMZA</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>chef projet</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>643.98</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>2101.08</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>4269.94</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>N°006</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K6"/>
+  <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
seeing how much paiment file for an employee
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,11 +494,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -837,8 +837,53 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>PIERE</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>JHON JACK</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chef projet </t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>4800</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>492.87</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1524.98</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>3351.14</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Aout 2026</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>N°007</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:K8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixing the number of payslip
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,441 +494,437 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Prenom</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Salaire Base</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Heures Sup</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Prime</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CNSS</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>IR</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Salaire Net</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Periode</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Bulletin</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>ABIDI</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">ABIDI </t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>MED aziz</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>developpeur</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Developpeur</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>2900</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>480</v>
-      </c>
       <c r="G2" s="3" t="n">
-        <v>311.11</v>
+        <v>500</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>831.98</v>
+        <v>312.95</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2245.91</v>
+        <v>838.98</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>2257.07</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>N°001</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
+      <c r="A3" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">BRAHMI </t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
           <t>HAMZA</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>chef projet</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
         <v>6000</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="F3" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="H3" s="7" t="n">
         <v>644.25</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="I3" s="8" t="n">
         <v>2102.13</v>
       </c>
-      <c r="I3" s="8" t="n">
-        <v>4271.61</v>
-      </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
+          <t>4271.61</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>N°002</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>KADRI</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NACER</t>
+          <t>BEN SLEMA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cheft projet </t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>6000</v>
+          <t>AHMED</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>responsable logistique</t>
+        </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6</v>
+        <v>4500</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>500</v>
+        <v>8</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>597.53</v>
+        <v>560</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1923.98</v>
+        <v>465.61</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3987.49</v>
+        <v>1421.03</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>3185.36</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>N°003</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>BEN ISSA</t>
-        </is>
+      <c r="A5" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>MARIEM</t>
+          <t>KADRI</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>RH</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>5800</v>
+          <t>NACER</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>CHEF PROJET</t>
+        </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>7</v>
+        <v>6000</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>670</v>
+        <v>6</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>594.91</v>
+        <v>500</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1914.01</v>
+        <v>597.53</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>3971.58</v>
+        <v>1923.98</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
+          <t>3987.49</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>N°004</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>AL AZIZ</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MOSTAFA</t>
+          <t>BESBES</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>RESPONSABLE LOGISTIQUE</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>4500</v>
+          <t>MARIEM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>RH</t>
+        </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>9</v>
+        <v>5000</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>560</v>
+        <v>6</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>465.75</v>
+        <v>500</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1421.56</v>
+        <v>505.73</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3186.19</v>
+        <v>1573.98</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>3429.29</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>N°005</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
+      <c r="A7" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>ABIDI</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>chef projet</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>6000</v>
+          <t>MED aziz</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Developpeur</t>
+        </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>10</v>
+        <v>2900</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1000</v>
+        <v>8</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>643.98</v>
+        <v>700</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>2101.08</v>
+        <v>331.58</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>4269.94</v>
+        <v>910.03</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
+          <t>2370.39</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>N°006</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>PIERE</t>
-        </is>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>JHON JACK</t>
+          <t>BRAHMI</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>HAMZA</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">chef projet </t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>4800</v>
-      </c>
       <c r="E8" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>560</v>
-      </c>
       <c r="G8" s="3" t="n">
-        <v>492.87</v>
+        <v>500</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>1524.98</v>
+        <v>597.53</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3351.14</v>
+        <v>1923.98</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
+          <t>3987.49</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
           <t>Aout 2026</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>N°007</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>ABIDI</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>MED aziz</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>developpeur</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>2900</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>640</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>325.8</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>887.98</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>2335.22</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="K9" s="9" t="inlineStr">
-        <is>
-          <t>N°008</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K9"/>
+  <autoFilter ref="A1:L8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixing the historic payslip and the comparison
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -579,7 +579,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABIDI </t>
+          <t>ABIDI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Developpeur</t>
+          <t>developpeur</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -639,7 +639,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>chef projet</t>
+          <t xml:space="preserve">chef projet </t>
         </is>
       </c>
       <c r="E3" s="6" t="n">
@@ -679,37 +679,37 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BEN SLEMA</t>
+          <t xml:space="preserve">KADRI </t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>AHMED</t>
+          <t>NACER</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>responsable logistique</t>
+          <t xml:space="preserve">chef projet </t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4500</v>
+        <v>6000</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>560</v>
+        <v>500</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>465.61</v>
+        <v>597.53</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1421.03</v>
+        <v>1923.98</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>3185.36</t>
+          <t>3987.49</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -729,37 +729,37 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>KADRI</t>
+          <t>BESBES</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>NACER</t>
+          <t>MARIEM</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>CHEF PROJET</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>6000</v>
+        <v>4500</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>597.53</v>
+        <v>487.78</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>1923.98</v>
+        <v>1505.56</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>3987.49</t>
+          <t>3320.16</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr">
@@ -779,37 +779,37 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>BESBES</t>
+          <t>BEN SLEMA</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MARIEM</t>
+          <t>BILEL</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>technisien supérieur</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>500</v>
+        <v>260</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>505.73</v>
+        <v>162.12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1573.98</v>
+        <v>300.63</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>3429.29</t>
+          <t>1303.25</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -829,37 +829,37 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>ABIDI</t>
+          <t>HWAWI</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>MED aziz</t>
+          <t>HADIL</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Developpeur</t>
+          <t>responsable logistique</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2900</v>
+        <v>3800</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>700</v>
+        <v>480</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>331.58</v>
+        <v>393.45</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>910.03</v>
+        <v>1145.93</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>2370.39</t>
+          <t>2746.61</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
@@ -870,61 +870,11 @@
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>N°006</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>HAMZA</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>500</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>597.53</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>1923.98</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>3987.49</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>N°007</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
see all the pay slip for the same employee
</commit_message>
<xml_diff>
--- a/saves/employes.xlsx
+++ b/saves/employes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employes'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -596,20 +596,20 @@
         <v>2900</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>312.95</v>
+        <v>359.67</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>838.98</v>
+        <v>1017.13</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2257.07</t>
+          <t>2541.19</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>N°001</t>
+          <t>N°006</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRAHMI </t>
+          <t>BRAHMI</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">chef projet </t>
+          <t xml:space="preserve">CHEF PROJET </t>
         </is>
       </c>
       <c r="E3" s="6" t="n">
@@ -684,7 +684,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>NACER</t>
+          <t xml:space="preserve"> NACER</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>BESBES</t>
+          <t xml:space="preserve">BESBES </t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -739,27 +739,27 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t xml:space="preserve">RH </t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
         <v>4500</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>487.78</v>
+        <v>436.05</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>1505.56</v>
+        <v>1308.33</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>3320.16</t>
+          <t>3005.62</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr">
@@ -779,37 +779,37 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>BEN SLEMA</t>
+          <t>ABIDI</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>BILEL</t>
+          <t>MED aziz</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>technisien supérieur</t>
+          <t>developpeur</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1500</v>
+        <v>2900</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>260</v>
+        <v>1000</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>162.12</v>
+        <v>359.67</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>300.63</v>
+        <v>1017.13</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>1303.25</t>
+          <t>2541.19</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -820,61 +820,11 @@
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>N°005</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>HWAWI</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>HADIL</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>responsable logistique</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>3800</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>480</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>393.45</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>1145.93</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>2746.61</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>N°006</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>